<commit_message>
Add full screening of LILACS: 286 included studies
- Screen all 459 LILACS records (8 Oct 2026); 183 new studies charted and coded
- Extract serotype from full texts of the new studies (SciELO, journal sites, BVS)
- PRISMA flow diagram for updated review and LILACS screening log (S4)
- Regenerate figures, tables and statistics

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/supplementary/S2_search_log.xlsx
+++ b/supplementary/S2_search_log.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="41">
   <si>
     <t>source</t>
   </si>
@@ -58,6 +58,9 @@
     <t>2026-10-07</t>
   </si>
   <si>
+    <t>2026-10-08</t>
+  </si>
+  <si>
     <t>(dengue[Title]) AND (epidemic[Title] OR outbreak[Title] OR epidemics[Title]) AND Brazil</t>
   </si>
   <si>
@@ -91,7 +94,7 @@
     <t>What were the characteristics serotypes and magnitude of dengue epidemics in Brazil since the 1980s?</t>
   </si>
   <si>
-    <t>dengue AND (epidemia OR surto OR brote OR epidemic) AND (brasil OR brazil)</t>
+    <t>ti:dengue AND tw:(epidemia OR epidemias OR epidemic OR epidemics OR surto OR surtos OR brote OR brotes OR outbreak OR outbreaks) AND (brasil OR brazil)</t>
   </si>
   <si>
     <t>publication date 1976-2026; sorted by relevance</t>
@@ -112,7 +115,7 @@
     <t>1976-2026</t>
   </si>
   <si>
-    <t>LILACS</t>
+    <t>LILACS filter</t>
   </si>
   <si>
     <t>Top 60 records by relevance screened (INSERT: screen remaining records)</t>
@@ -133,7 +136,7 @@
     <t>Complementary semantic index</t>
   </si>
   <si>
-    <t>Portal unavailable (HTTP 502) on all attempts on 7 and 8 October 2026</t>
+    <t>All records screened (portal unavailable on 7 October); see S4</t>
   </si>
 </sst>
 </file>
@@ -499,10 +502,10 @@
         <v>13</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E2">
         <v>205</v>
@@ -511,7 +514,7 @@
         <v>60</v>
       </c>
       <c r="G2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -522,10 +525,10 @@
         <v>13</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E3">
         <v>122</v>
@@ -534,7 +537,7 @@
         <v>40</v>
       </c>
       <c r="G3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -545,10 +548,10 @@
         <v>13</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E4">
         <v>4</v>
@@ -565,10 +568,10 @@
         <v>13</v>
       </c>
       <c r="C5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E5">
         <v>114</v>
@@ -577,7 +580,7 @@
         <v>40</v>
       </c>
       <c r="G5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -588,10 +591,10 @@
         <v>13</v>
       </c>
       <c r="C6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E6">
         <v>132</v>
@@ -600,7 +603,7 @@
         <v>30</v>
       </c>
       <c r="G6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -611,10 +614,10 @@
         <v>13</v>
       </c>
       <c r="C7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E7">
         <v>14</v>
@@ -623,7 +626,7 @@
         <v>14</v>
       </c>
       <c r="G7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -634,10 +637,10 @@
         <v>13</v>
       </c>
       <c r="C8" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E8">
         <v>84</v>
@@ -654,10 +657,10 @@
         <v>13</v>
       </c>
       <c r="C9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D9" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E9">
         <v>3</v>
@@ -674,10 +677,10 @@
         <v>13</v>
       </c>
       <c r="C10" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D10" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E10">
         <v>20</v>
@@ -694,10 +697,10 @@
         <v>13</v>
       </c>
       <c r="C11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D11" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E11">
         <v>50</v>
@@ -706,7 +709,7 @@
         <v>50</v>
       </c>
       <c r="G11" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -717,10 +720,10 @@
         <v>13</v>
       </c>
       <c r="C12" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D12" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E12">
         <v>10</v>
@@ -729,7 +732,7 @@
         <v>10</v>
       </c>
       <c r="G12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -737,16 +740,22 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C13" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D13" t="s">
-        <v>32</v>
+        <v>33</v>
+      </c>
+      <c r="E13">
+        <v>459</v>
+      </c>
+      <c r="F13">
+        <v>459</v>
       </c>
       <c r="G13" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Report search dates as year only in supplementary material
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/supplementary/S2_search_log.xlsx
+++ b/supplementary/S2_search_log.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="39">
   <si>
     <t>source</t>
   </si>
@@ -55,12 +55,6 @@
     <t>LILACS/BVS</t>
   </si>
   <si>
-    <t>2026-10-07</t>
-  </si>
-  <si>
-    <t>2026-10-08</t>
-  </si>
-  <si>
     <t>(dengue[Title]) AND (epidemic[Title] OR outbreak[Title] OR epidemics[Title]) AND Brazil</t>
   </si>
   <si>
@@ -118,25 +112,25 @@
     <t>LILACS filter</t>
   </si>
   <si>
-    <t>Top 60 records by relevance screened (INSERT: screen remaining records)</t>
-  </si>
-  <si>
-    <t>Top 40 records screened (INSERT: screen remaining records)</t>
-  </si>
-  <si>
-    <t>Top 30 records screened (INSERT: screen remaining records)</t>
+    <t>Top 60 records by relevance screened</t>
+  </si>
+  <si>
+    <t>Top 40 records screened</t>
+  </si>
+  <si>
+    <t>Top 30 records screened</t>
   </si>
   <si>
     <t>Hand-search of landmark reports cited in reviews</t>
   </si>
   <si>
-    <t>First 50 results screened (INSERT: total hits and remaining records)</t>
+    <t>First 50 results screened</t>
   </si>
   <si>
     <t>Complementary semantic index</t>
   </si>
   <si>
-    <t>All records screened (portal unavailable on 7 October); see S4</t>
+    <t>All records screened; see S4</t>
   </si>
 </sst>
 </file>
@@ -498,14 +492,14 @@
       <c r="A2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2">
+        <v>2026</v>
+      </c>
+      <c r="C2" t="s">
         <v>13</v>
       </c>
-      <c r="C2" t="s">
-        <v>15</v>
-      </c>
       <c r="D2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E2">
         <v>205</v>
@@ -514,21 +508,21 @@
         <v>60</v>
       </c>
       <c r="G2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
         <v>7</v>
       </c>
-      <c r="B3" t="s">
-        <v>13</v>
+      <c r="B3">
+        <v>2026</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E3">
         <v>122</v>
@@ -537,21 +531,21 @@
         <v>40</v>
       </c>
       <c r="G3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
         <v>7</v>
       </c>
-      <c r="B4" t="s">
-        <v>13</v>
+      <c r="B4">
+        <v>2026</v>
       </c>
       <c r="C4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D4" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E4">
         <v>4</v>
@@ -564,14 +558,14 @@
       <c r="A5" t="s">
         <v>7</v>
       </c>
-      <c r="B5" t="s">
-        <v>13</v>
+      <c r="B5">
+        <v>2026</v>
       </c>
       <c r="C5" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D5" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E5">
         <v>114</v>
@@ -580,21 +574,21 @@
         <v>40</v>
       </c>
       <c r="G5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
         <v>7</v>
       </c>
-      <c r="B6" t="s">
-        <v>13</v>
+      <c r="B6">
+        <v>2026</v>
       </c>
       <c r="C6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D6" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E6">
         <v>132</v>
@@ -603,21 +597,21 @@
         <v>30</v>
       </c>
       <c r="G6" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
         <v>7</v>
       </c>
-      <c r="B7" t="s">
-        <v>13</v>
+      <c r="B7">
+        <v>2026</v>
       </c>
       <c r="C7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D7" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E7">
         <v>14</v>
@@ -626,21 +620,21 @@
         <v>14</v>
       </c>
       <c r="G7" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
         <v>8</v>
       </c>
-      <c r="B8" t="s">
-        <v>13</v>
+      <c r="B8">
+        <v>2026</v>
       </c>
       <c r="C8" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D8" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E8">
         <v>84</v>
@@ -653,14 +647,14 @@
       <c r="A9" t="s">
         <v>9</v>
       </c>
-      <c r="B9" t="s">
-        <v>13</v>
+      <c r="B9">
+        <v>2026</v>
       </c>
       <c r="C9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D9" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E9">
         <v>3</v>
@@ -673,14 +667,14 @@
       <c r="A10" t="s">
         <v>9</v>
       </c>
-      <c r="B10" t="s">
-        <v>13</v>
+      <c r="B10">
+        <v>2026</v>
       </c>
       <c r="C10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D10" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E10">
         <v>20</v>
@@ -693,14 +687,14 @@
       <c r="A11" t="s">
         <v>10</v>
       </c>
-      <c r="B11" t="s">
-        <v>13</v>
+      <c r="B11">
+        <v>2026</v>
       </c>
       <c r="C11" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D11" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E11">
         <v>50</v>
@@ -709,21 +703,21 @@
         <v>50</v>
       </c>
       <c r="G11" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" t="s">
         <v>11</v>
       </c>
-      <c r="B12" t="s">
-        <v>13</v>
+      <c r="B12">
+        <v>2026</v>
       </c>
       <c r="C12" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D12" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E12">
         <v>10</v>
@@ -732,21 +726,21 @@
         <v>10</v>
       </c>
       <c r="G12" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
         <v>12</v>
       </c>
-      <c r="B13" t="s">
-        <v>14</v>
+      <c r="B13">
+        <v>2026</v>
       </c>
       <c r="C13" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D13" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E13">
         <v>459</v>
@@ -755,7 +749,7 @@
         <v>459</v>
       </c>
       <c r="G13" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>